<commit_message>
added changes for 6m band support also got rid of a Serial.End() that seemed to abort things now with new ide? will have to see if ALLOW_USB_DISABLE_MODE might work during test didn't test with sdr yet
</commit_message>
<xml_diff>
--- a/tracker/wspr_calc_direct_shift.xlsx
+++ b/tracker/wspr_calc_direct_shift.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="48">
   <si>
     <t xml:space="preserve">Note how it’s independent of the u4b frequency bin within the band.</t>
   </si>
@@ -42,6 +42,9 @@
     <t xml:space="preserve">20M </t>
   </si>
   <si>
+    <t xml:space="preserve">6M?</t>
+  </si>
+  <si>
     <t xml:space="preserve">will work for 25 and 27 also</t>
   </si>
   <si>
@@ -72,19 +75,28 @@
     <t xml:space="preserve">20M divider</t>
   </si>
   <si>
+    <t xml:space="preserve">6M divider</t>
+  </si>
+  <si>
     <t xml:space="preserve">That imply pll min/max</t>
   </si>
   <si>
     <t xml:space="preserve">10M mult</t>
   </si>
   <si>
+    <t xml:space="preserve">12M mult</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15M mult</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17M mult</t>
+  </si>
+  <si>
     <t xml:space="preserve">20M mult</t>
   </si>
   <si>
-    <t xml:space="preserve">15M mult</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17M mult</t>
+    <t xml:space="preserve">6M mult</t>
   </si>
   <si>
     <t xml:space="preserve">pll freq max</t>
@@ -263,7 +275,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -289,10 +301,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -503,7 +511,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.67"/>
@@ -540,14 +548,21 @@
         <v>5</v>
       </c>
       <c r="L2" s="2"/>
+      <c r="M2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>26000000</v>
@@ -556,10 +571,12 @@
       <c r="H4" s="4"/>
       <c r="J4" s="4"/>
       <c r="L4" s="4"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">12000/8192</f>
@@ -569,10 +586,12 @@
       <c r="H5" s="4"/>
       <c r="J5" s="4"/>
       <c r="L5" s="4"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>1048575</v>
@@ -581,171 +600,206 @@
       <c r="H6" s="4"/>
       <c r="J6" s="4"/>
       <c r="L6" s="4"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>20</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>24</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>28</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>36</v>
       </c>
+      <c r="M7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>19</v>
       </c>
+      <c r="M8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">(D8+1) * D4</f>
         <v>520000000</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">(F8+1) * D4</f>
         <v>520000000</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">(H8+1) * D4</f>
         <v>520000000</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J9" s="4" t="n">
         <f aca="false">(J8+1) * D4</f>
         <v>520000000</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="L9" s="4" t="n">
         <f aca="false">(L8+1) * D4</f>
         <v>520000000</v>
       </c>
+      <c r="M9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <f aca="false">(N8+1) * D4</f>
+        <v>832000000</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D10" s="4" t="n">
         <f aca="false">D8*D4</f>
         <v>494000000</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F10" s="4" t="n">
         <f aca="false">F8*D4</f>
         <v>494000000</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H10" s="4" t="n">
         <f aca="false">H8 * D4</f>
         <v>494000000</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="J10" s="4" t="n">
         <f aca="false">J8*D4</f>
         <v>494000000</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="L10" s="4" t="n">
         <f aca="false">L8*D4</f>
         <v>494000000</v>
       </c>
+      <c r="M10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <f aca="false">N8*D4</f>
+        <v>806000000</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G11" s="5"/>
+      <c r="M11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -784,6 +838,16 @@
         <f aca="false">MIN(1*(D4/L7)/D5, D6)</f>
         <v>493037.037037037</v>
       </c>
+      <c r="M13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <f aca="false">MIN(1*(D4/N7)/D5, D6)</f>
+        <v>1048575</v>
+      </c>
+      <c r="O13" s="1" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C14" s="1" t="n">
@@ -796,21 +860,21 @@
       <c r="E14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="7" t="n">
         <f aca="false">MIN(2*(D4/F7)/D5, D6)</f>
         <v>1048575</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="7" t="n">
         <f aca="false">MIN(2*(D4/H7)/D5, D6)</f>
         <v>1048575</v>
       </c>
       <c r="I14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="7" t="n">
         <f aca="false">MIN(2*(D4/J7)/D5,D6)</f>
         <v>1048575</v>
       </c>
@@ -821,6 +885,16 @@
         <f aca="false">MIN(2*(D4/L7)/D5, D6)</f>
         <v>986074.074074074</v>
       </c>
+      <c r="M14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <f aca="false">MIN(2*(D4/N7)/D5, D6)</f>
+        <v>1048575</v>
+      </c>
+      <c r="O14" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C15" s="1" t="n">
@@ -847,107 +921,118 @@
       <c r="I15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="J15" s="8" t="n">
+      <c r="J15" s="7" t="n">
         <f aca="false">MIN(3*(D4/J7)/D5, D6)</f>
         <v>1048575</v>
       </c>
       <c r="K15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="L15" s="8" t="n">
+      <c r="L15" s="7" t="n">
         <f aca="false">MIN(3*(D4/L7)/D5,D6)</f>
         <v>1048575</v>
       </c>
+      <c r="M15" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="N15" s="7" t="n">
+        <f aca="false">MIN(3*(D4/N7)/D5,D6)</f>
+        <v>1048575</v>
+      </c>
+      <c r="O15" s="1" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D18" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J22" s="9" t="s">
-        <v>25</v>
+      <c r="J22" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E29" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D32" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H32" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I32" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="J32" s="10" t="s">
+      <c r="E32" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K32" s="10" t="s">
+      <c r="F32" s="9"/>
+      <c r="G32" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L32" s="10" t="n">
+      <c r="H32" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="J32" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="K32" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="L32" s="9" t="n">
         <v>96467329</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E33" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E34" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E35" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E36" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E38" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E39" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M2:N2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A8:B8"/>
@@ -1011,11 +1096,11 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>26000000</v>
@@ -1027,7 +1112,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>15.625</v>
@@ -1039,7 +1124,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>1048575</v>
@@ -1051,35 +1136,35 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>32</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>42</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>50</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>64</v>
@@ -1087,35 +1172,35 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>34</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>34</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>34</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>34</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>34</v>
@@ -1123,35 +1208,35 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">(D8+1) * D4</f>
         <v>910000000</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">(F8+1) * D4</f>
         <v>910000000</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">(H8+1) * D4</f>
         <v>910000000</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J9" s="4" t="n">
         <f aca="false">(J8+1) * D4</f>
         <v>910000000</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="L9" s="4" t="n">
         <f aca="false">(L8+1) * D4</f>
@@ -1160,35 +1245,35 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D10" s="4" t="n">
         <f aca="false">D8*D4</f>
         <v>884000000</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F10" s="4" t="n">
         <f aca="false">F8*D4</f>
         <v>884000000</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H10" s="4" t="n">
         <f aca="false">H8 * D4</f>
         <v>884000000</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="J10" s="4" t="n">
         <f aca="false">J8*D4</f>
         <v>884000000</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="L10" s="4" t="n">
         <f aca="false">L8*D4</f>
@@ -1200,54 +1285,54 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="10" t="n">
         <f aca="false">MIN(1*(D4/D7)/D5, D6)</f>
         <v>52000</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="11" t="n">
         <f aca="false">MIN(1*(D4/F7)/D5, D6)</f>
         <v>46222.2222222222</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="12" t="n">
+      <c r="H13" s="11" t="n">
         <f aca="false">MIN((D4/H7)/D5, D6)</f>
         <v>39619.0476190476</v>
       </c>
       <c r="I13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="J13" s="12" t="n">
+      <c r="J13" s="11" t="n">
         <f aca="false">MIN(1*(D4/J7)/D5, D6)</f>
         <v>33280</v>
       </c>
       <c r="K13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="L13" s="12" t="n">
+      <c r="L13" s="11" t="n">
         <f aca="false">MIN(1*(D4/L7)/D5, D6)</f>
         <v>26000</v>
       </c>
@@ -1256,35 +1341,35 @@
       <c r="C14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="11" t="n">
         <f aca="false">MIN(2*(D4/D7) / D5, D6)</f>
         <v>104000</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="10" t="n">
         <f aca="false">MIN(2*(D4/F7)/D5, D6)</f>
         <v>92444.4444444445</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="11" t="n">
+      <c r="H14" s="10" t="n">
         <f aca="false">MIN(2*(D4/H7)/D5, D6)</f>
         <v>79238.0952380952</v>
       </c>
       <c r="I14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="J14" s="11" t="n">
+      <c r="J14" s="10" t="n">
         <f aca="false">MIN(2*(D4/J7)/D5,D6)</f>
         <v>66560</v>
       </c>
       <c r="K14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="L14" s="12" t="n">
+      <c r="L14" s="11" t="n">
         <f aca="false">MIN(2*(D4/L7)/D5, D6)</f>
         <v>52000</v>
       </c>
@@ -1293,117 +1378,117 @@
       <c r="C15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="11" t="n">
         <f aca="false">MIN(3*(D4/D7)/D5, D6)</f>
         <v>156000</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="11" t="n">
         <f aca="false">MIN(3*(D6/F7)/D5, D6)</f>
         <v>5592.4</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="H15" s="12" t="n">
+      <c r="H15" s="11" t="n">
         <f aca="false">MIN(3*(D4/H7)/D5, D6)</f>
         <v>118857.142857143</v>
       </c>
       <c r="I15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="11" t="n">
         <f aca="false">MIN(3*(D4/J7)/D5, D6)</f>
         <v>99840</v>
       </c>
       <c r="K15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="L15" s="11" t="n">
+      <c r="L15" s="10" t="n">
         <f aca="false">MIN(3*(D4/L7)/D5,D6)</f>
         <v>78000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D18" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J22" s="9"/>
+      <c r="J22" s="8"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E29" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D32" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H32" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I32" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="J32" s="10" t="s">
+      <c r="E32" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K32" s="10" t="s">
+      <c r="F32" s="9"/>
+      <c r="G32" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L32" s="10" t="n">
+      <c r="H32" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="J32" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="K32" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="L32" s="9" t="n">
         <v>96467329</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E33" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E34" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E35" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E36" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E38" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E39" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1476,11 +1561,11 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>26000000</v>
@@ -1492,7 +1577,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>15.625</v>
@@ -1504,7 +1589,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>1048575</v>
@@ -1516,35 +1601,35 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>42</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>50</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>64</v>
@@ -1552,35 +1637,35 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>34</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>34</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>34</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>34</v>
@@ -1588,35 +1673,35 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">(D8+1) * D4</f>
         <v>520000000</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">(F8+1) * D4</f>
         <v>910000000</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">(H8+1) * D4</f>
         <v>910000000</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J9" s="4" t="n">
         <f aca="false">(J8+1) * D4</f>
         <v>910000000</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="L9" s="4" t="n">
         <f aca="false">(L8+1) * D4</f>
@@ -1625,35 +1710,35 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D10" s="4" t="n">
         <f aca="false">D8*D4</f>
         <v>494000000</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F10" s="4" t="n">
         <f aca="false">F8*D4</f>
         <v>884000000</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H10" s="4" t="n">
         <f aca="false">H8 * D4</f>
         <v>884000000</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="J10" s="4" t="n">
         <f aca="false">J8*D4</f>
         <v>884000000</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="L10" s="4" t="n">
         <f aca="false">L8*D4</f>
@@ -1665,26 +1750,26 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="12" t="n">
         <f aca="false">MIN(1*(D4/D7)/D5, D6)</f>
         <v>92444.4444444445</v>
       </c>
@@ -1728,21 +1813,21 @@
       <c r="E14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="12" t="n">
         <f aca="false">MIN(2*(D4/F7)/D5, D6)</f>
         <v>92444.4444444445</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="13" t="n">
+      <c r="H14" s="12" t="n">
         <f aca="false">MIN(2*(D4/H7)/D5, D6)</f>
         <v>79238.0952380952</v>
       </c>
       <c r="I14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="J14" s="13" t="n">
+      <c r="J14" s="12" t="n">
         <f aca="false">MIN(2*(D4/J7)/D5,D6)</f>
         <v>66560</v>
       </c>
@@ -1786,7 +1871,7 @@
       <c r="K15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="L15" s="13" t="n">
+      <c r="L15" s="12" t="n">
         <f aca="false">MIN(3*(D4/L7)/D5,D6)</f>
         <v>78000</v>
       </c>
@@ -1796,87 +1881,87 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D18" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D21" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J22" s="9"/>
+      <c r="J22" s="8"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E29" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D32" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H32" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I32" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="J32" s="10" t="s">
+      <c r="E32" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K32" s="10" t="s">
+      <c r="F32" s="9"/>
+      <c r="G32" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L32" s="10" t="n">
+      <c r="H32" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="J32" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="K32" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="L32" s="9" t="n">
         <v>96467329</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E33" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E34" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E35" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E36" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E38" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E39" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>